<commit_message>
Atualiza datasets e rankings de scouts
</commit_message>
<xml_diff>
--- a/scouts/datasets_scouts/pesos_times.xlsx
+++ b/scouts/datasets_scouts/pesos_times.xlsx
@@ -473,29 +473,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>SAO</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>56</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>41</v>
+        <v>4</v>
       </c>
       <c r="G2" t="n">
-        <v>204.2</v>
+        <v>199.4</v>
       </c>
       <c r="H2" t="n">
-        <v>153.4</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3">
@@ -505,389 +505,389 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="E3" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="G3" t="n">
-        <v>187.8</v>
+        <v>200.4</v>
       </c>
       <c r="H3" t="n">
-        <v>141.4</v>
+        <v>149.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>CAP</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="D4" t="n">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>149.4</v>
+        <v>183.2</v>
       </c>
       <c r="H4" t="n">
-        <v>110.2</v>
+        <v>140.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MIR</t>
+          <t>RBB</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="D5" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>150.2</v>
+        <v>148.2</v>
       </c>
       <c r="H5" t="n">
-        <v>104.8</v>
+        <v>114.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BOT</t>
+          <t>BAH</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>151.2</v>
+        <v>184.4</v>
       </c>
       <c r="H6" t="n">
-        <v>113.6</v>
+        <v>140.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BAH</t>
+          <t>FLU</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C7" t="n">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="E7" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>159.4</v>
+        <v>176.6</v>
       </c>
       <c r="H7" t="n">
-        <v>102.8</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FLU</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="D8" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>140.6</v>
+        <v>209.6</v>
       </c>
       <c r="H8" t="n">
-        <v>92.40000000000001</v>
+        <v>154.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>VAS</t>
+          <t>GRE</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="D9" t="n">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="E9" t="n">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="F9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>136.4</v>
+        <v>188.6</v>
       </c>
       <c r="H9" t="n">
-        <v>96.59999999999999</v>
+        <v>133.4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SAO</t>
+          <t>MIR</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C10" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="D10" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="E10" t="n">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="F10" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>124.6</v>
+        <v>176.4</v>
       </c>
       <c r="H10" t="n">
-        <v>83.19999999999999</v>
+        <v>126.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>CHA</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="D11" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="E11" t="n">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="F11" t="n">
-        <v>-4</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>134.4</v>
+        <v>128.8</v>
       </c>
       <c r="H11" t="n">
-        <v>90.2</v>
+        <v>94.40000000000001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RBB</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="D12" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="E12" t="n">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>-10</v>
+        <v>-2</v>
       </c>
       <c r="G12" t="n">
-        <v>120</v>
+        <v>127.8</v>
       </c>
       <c r="H12" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GRE</t>
+          <t>FLA</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="F13" t="n">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>110.4</v>
+        <v>174</v>
       </c>
       <c r="H13" t="n">
-        <v>72.39999999999999</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CEA</t>
+          <t>CFC</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E14" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G14" t="n">
-        <v>99.59999999999999</v>
+        <v>89.39999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>67.40000000000001</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>REM</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="E15" t="n">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="F15" t="n">
-        <v>-6</v>
+        <v>-2</v>
       </c>
       <c r="G15" t="n">
-        <v>136.8</v>
+        <v>127.6</v>
       </c>
       <c r="H15" t="n">
-        <v>86.59999999999999</v>
+        <v>90.19999999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAM</t>
+          <t>BOT</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E16" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="F16" t="n">
-        <v>-6</v>
+        <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="H16" t="n">
-        <v>74.39999999999999</v>
+        <v>89.60000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -897,137 +897,137 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="C17" t="n">
-        <v>31</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="E17" t="n">
-        <v>43</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>-16</v>
+        <v>-3</v>
       </c>
       <c r="G17" t="n">
-        <v>110.4</v>
+        <v>116.6</v>
       </c>
       <c r="H17" t="n">
-        <v>62</v>
+        <v>81.60000000000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="E18" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="F18" t="n">
-        <v>-12</v>
+        <v>-3</v>
       </c>
       <c r="G18" t="n">
-        <v>102.2</v>
+        <v>102.8</v>
       </c>
       <c r="H18" t="n">
-        <v>63.59999999999999</v>
+        <v>73.40000000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>JUV</t>
+          <t>CRU</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="E19" t="n">
-        <v>53</v>
+        <v>9</v>
       </c>
       <c r="F19" t="n">
-        <v>-30</v>
+        <v>-5</v>
       </c>
       <c r="G19" t="n">
-        <v>94</v>
+        <v>103.8</v>
       </c>
       <c r="H19" t="n">
-        <v>45</v>
+        <v>71.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FOR</t>
+          <t>CAM</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="E20" t="n">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="F20" t="n">
-        <v>-18</v>
+        <v>-2</v>
       </c>
       <c r="G20" t="n">
-        <v>91.80000000000001</v>
+        <v>153.6</v>
       </c>
       <c r="H20" t="n">
-        <v>53.4</v>
+        <v>103.2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>VAS</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="F21" t="n">
-        <v>-23</v>
+        <v>-3</v>
       </c>
       <c r="G21" t="n">
-        <v>73</v>
+        <v>104.2</v>
       </c>
       <c r="H21" t="n">
-        <v>42.2</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza scouts e adiciona novas visoes
</commit_message>
<xml_diff>
--- a/scouts/datasets_scouts/pesos_times.xlsx
+++ b/scouts/datasets_scouts/pesos_times.xlsx
@@ -477,557 +477,557 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D2" t="n">
         <v>10</v>
       </c>
-      <c r="D2" t="n">
-        <v>6</v>
-      </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G2" t="n">
-        <v>199.4</v>
+        <v>98.98785239514096</v>
       </c>
       <c r="H2" t="n">
-        <v>149</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PAL</t>
+          <t>FLU</t>
         </is>
       </c>
       <c r="B3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F3" t="n">
         <v>4</v>
       </c>
-      <c r="C3" t="n">
-        <v>10</v>
-      </c>
-      <c r="D3" t="n">
-        <v>12</v>
-      </c>
-      <c r="E3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F3" t="n">
-        <v>7</v>
-      </c>
       <c r="G3" t="n">
-        <v>200.4</v>
+        <v>86.73206509282605</v>
       </c>
       <c r="H3" t="n">
-        <v>149.8</v>
+        <v>79.35595418197536</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAP</t>
+          <t>PAL</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C4" t="n">
+        <v>13</v>
+      </c>
+      <c r="D4" t="n">
+        <v>14</v>
+      </c>
+      <c r="E4" t="n">
         <v>7</v>
       </c>
-      <c r="D4" t="n">
-        <v>4</v>
-      </c>
-      <c r="E4" t="n">
-        <v>3</v>
-      </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G4" t="n">
-        <v>183.2</v>
+        <v>100</v>
       </c>
       <c r="H4" t="n">
-        <v>140.4</v>
+        <v>85.19126864058786</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RBB</t>
+          <t>BAH</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>148.2</v>
+        <v>60.33554893421957</v>
       </c>
       <c r="H5" t="n">
-        <v>114.8</v>
+        <v>97.08666522584829</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BAH</t>
+          <t>FLA</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" t="n">
         <v>4</v>
       </c>
-      <c r="E6" t="n">
-        <v>2</v>
-      </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G6" t="n">
-        <v>184.4</v>
+        <v>79.08228283291314</v>
       </c>
       <c r="H6" t="n">
-        <v>140.8</v>
+        <v>92.93710827750164</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FLU</t>
+          <t>CFC</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" t="n">
-        <v>176.6</v>
+        <v>50.72381388952556</v>
       </c>
       <c r="H7" t="n">
-        <v>127</v>
+        <v>83.16835962826886</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>RBB</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D8" t="n">
         <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="G8" t="n">
-        <v>209.6</v>
+        <v>51.31423332569334</v>
       </c>
       <c r="H8" t="n">
-        <v>154.6</v>
+        <v>56.78409336503134</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GRE</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>188.6</v>
+        <v>48.78019711207885</v>
       </c>
       <c r="H9" t="n">
-        <v>133.4</v>
+        <v>67.90144802247679</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MIR</t>
+          <t>GRE</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>176.4</v>
+        <v>70.30300252120101</v>
       </c>
       <c r="H10" t="n">
-        <v>126.2</v>
+        <v>45.45061594985953</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>CAP</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E11" t="n">
         <v>6</v>
       </c>
       <c r="F11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>128.8</v>
+        <v>52.68943387577356</v>
       </c>
       <c r="H11" t="n">
-        <v>94.40000000000001</v>
+        <v>60.35444132267128</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>VIT</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D12" t="n">
+        <v>7</v>
+      </c>
+      <c r="E12" t="n">
         <v>8</v>
       </c>
-      <c r="E12" t="n">
-        <v>10</v>
-      </c>
       <c r="F12" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="G12" t="n">
-        <v>127.8</v>
+        <v>61.39170295668119</v>
       </c>
       <c r="H12" t="n">
-        <v>91</v>
+        <v>38.9409984871407</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D13" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G13" t="n">
-        <v>174</v>
+        <v>52.39972495988999</v>
       </c>
       <c r="H13" t="n">
-        <v>127</v>
+        <v>37.32440025934731</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CFC</t>
+          <t>MIR</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E14" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>89.39999999999999</v>
+        <v>56.14027045610819</v>
       </c>
       <c r="H14" t="n">
-        <v>70</v>
+        <v>49.00367408688135</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>REM</t>
+          <t>CHA</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D15" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F15" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>127.6</v>
+        <v>57.09741003896402</v>
       </c>
       <c r="H15" t="n">
-        <v>90.19999999999999</v>
+        <v>44.95785606224335</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BOT</t>
+          <t>VAS</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="G16" t="n">
-        <v>131</v>
+        <v>47.40866376346551</v>
       </c>
       <c r="H16" t="n">
-        <v>89.60000000000001</v>
+        <v>39.64123622217419</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>VIT</t>
+          <t>CAM</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E17" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F17" t="n">
         <v>-3</v>
       </c>
       <c r="G17" t="n">
-        <v>116.6</v>
+        <v>52.91313316525327</v>
       </c>
       <c r="H17" t="n">
-        <v>81.60000000000001</v>
+        <v>30.85800734817376</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>BOT</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F18" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G18" t="n">
-        <v>102.8</v>
+        <v>48.91588356635343</v>
       </c>
       <c r="H18" t="n">
-        <v>73.40000000000001</v>
+        <v>31.70520855846121</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>REM</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E19" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F19" t="n">
         <v>-5</v>
       </c>
       <c r="G19" t="n">
-        <v>103.8</v>
+        <v>27.03002521201008</v>
       </c>
       <c r="H19" t="n">
-        <v>71.2</v>
+        <v>26.30213961530149</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAM</t>
+          <t>CRU</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E20" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F20" t="n">
-        <v>-2</v>
+        <v>-7</v>
       </c>
       <c r="G20" t="n">
-        <v>153.6</v>
+        <v>33.43295897318359</v>
       </c>
       <c r="H20" t="n">
-        <v>103.2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>VAS</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" t="n">
         <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F21" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="G21" t="n">
-        <v>104.2</v>
+        <v>20</v>
       </c>
       <c r="H21" t="n">
-        <v>71</v>
+        <v>36.85757510265831</v>
       </c>
     </row>
   </sheetData>

</xml_diff>